<commit_message>
Auto update ESO load data
</commit_message>
<xml_diff>
--- a/data/plexos_load_master.xlsx
+++ b/data/plexos_load_master.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA221"/>
+  <dimension ref="A1:AA222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18419,76 +18419,76 @@
         <v>8</v>
       </c>
       <c r="D217" t="n">
-        <v>3376</v>
+        <v>3282</v>
       </c>
       <c r="E217" t="n">
-        <v>3180</v>
+        <v>3112</v>
       </c>
       <c r="F217" t="n">
-        <v>3074</v>
+        <v>3022</v>
       </c>
       <c r="G217" t="n">
-        <v>3024</v>
+        <v>2979</v>
       </c>
       <c r="H217" t="n">
-        <v>3017</v>
+        <v>2974</v>
       </c>
       <c r="I217" t="n">
-        <v>3112</v>
+        <v>3067</v>
       </c>
       <c r="J217" t="n">
-        <v>3386</v>
+        <v>3338</v>
       </c>
       <c r="K217" t="n">
-        <v>3666</v>
+        <v>3614</v>
       </c>
       <c r="L217" t="n">
-        <v>3976</v>
+        <v>3916</v>
       </c>
       <c r="M217" t="n">
-        <v>4144</v>
+        <v>4074</v>
       </c>
       <c r="N217" t="n">
-        <v>4222</v>
+        <v>4142</v>
       </c>
       <c r="O217" t="n">
-        <v>4329</v>
+        <v>4249</v>
       </c>
       <c r="P217" t="n">
+        <v>4316</v>
+      </c>
+      <c r="Q217" t="n">
+        <v>4466</v>
+      </c>
+      <c r="R217" t="n">
         <v>4397</v>
       </c>
-      <c r="Q217" t="n">
-        <v>4549</v>
-      </c>
-      <c r="R217" t="n">
-        <v>4502</v>
-      </c>
       <c r="S217" t="n">
-        <v>4484</v>
+        <v>4350</v>
       </c>
       <c r="T217" t="n">
-        <v>4420</v>
+        <v>4278</v>
       </c>
       <c r="U217" t="n">
-        <v>4387</v>
+        <v>4242</v>
       </c>
       <c r="V217" t="n">
-        <v>4712</v>
+        <v>4526</v>
       </c>
       <c r="W217" t="n">
-        <v>4683</v>
+        <v>4504</v>
       </c>
       <c r="X217" t="n">
-        <v>4682</v>
+        <v>4550</v>
       </c>
       <c r="Y217" t="n">
-        <v>4388</v>
+        <v>4244</v>
       </c>
       <c r="Z217" t="n">
-        <v>4018</v>
+        <v>3930</v>
       </c>
       <c r="AA217" t="n">
-        <v>3676</v>
+        <v>3636</v>
       </c>
     </row>
     <row r="218">
@@ -18502,76 +18502,76 @@
         <v>9</v>
       </c>
       <c r="D218" t="n">
-        <v>3366</v>
+        <v>3276</v>
       </c>
       <c r="E218" t="n">
-        <v>3173</v>
+        <v>3107</v>
       </c>
       <c r="F218" t="n">
-        <v>3069</v>
+        <v>3019</v>
       </c>
       <c r="G218" t="n">
-        <v>3019</v>
+        <v>2976</v>
       </c>
       <c r="H218" t="n">
-        <v>3012</v>
+        <v>2971</v>
       </c>
       <c r="I218" t="n">
-        <v>3106</v>
+        <v>3064</v>
       </c>
       <c r="J218" t="n">
-        <v>3377</v>
+        <v>3333</v>
       </c>
       <c r="K218" t="n">
-        <v>3655</v>
+        <v>3608</v>
       </c>
       <c r="L218" t="n">
-        <v>3962</v>
+        <v>3907</v>
       </c>
       <c r="M218" t="n">
-        <v>4129</v>
+        <v>4065</v>
       </c>
       <c r="N218" t="n">
-        <v>4206</v>
+        <v>4133</v>
       </c>
       <c r="O218" t="n">
-        <v>4312</v>
+        <v>4239</v>
       </c>
       <c r="P218" t="n">
-        <v>4380</v>
+        <v>4305</v>
       </c>
       <c r="Q218" t="n">
-        <v>4530</v>
+        <v>4455</v>
       </c>
       <c r="R218" t="n">
-        <v>4483</v>
+        <v>4385</v>
       </c>
       <c r="S218" t="n">
-        <v>4465</v>
+        <v>4339</v>
       </c>
       <c r="T218" t="n">
-        <v>4401</v>
+        <v>4267</v>
       </c>
       <c r="U218" t="n">
-        <v>4369</v>
+        <v>4231</v>
       </c>
       <c r="V218" t="n">
-        <v>4699</v>
+        <v>4519</v>
       </c>
       <c r="W218" t="n">
-        <v>4671</v>
+        <v>4496</v>
       </c>
       <c r="X218" t="n">
-        <v>4670</v>
+        <v>4497</v>
       </c>
       <c r="Y218" t="n">
-        <v>4377</v>
+        <v>4237</v>
       </c>
       <c r="Z218" t="n">
-        <v>4009</v>
+        <v>3924</v>
       </c>
       <c r="AA218" t="n">
-        <v>3669</v>
+        <v>3632</v>
       </c>
     </row>
     <row r="219">
@@ -18585,76 +18585,76 @@
         <v>10</v>
       </c>
       <c r="D219" t="n">
-        <v>3372</v>
+        <v>3282</v>
       </c>
       <c r="E219" t="n">
-        <v>3177</v>
+        <v>3112</v>
       </c>
       <c r="F219" t="n">
-        <v>3072</v>
+        <v>3023</v>
       </c>
       <c r="G219" t="n">
-        <v>3023</v>
+        <v>2980</v>
       </c>
       <c r="H219" t="n">
-        <v>3015</v>
+        <v>2974</v>
       </c>
       <c r="I219" t="n">
-        <v>3110</v>
+        <v>3068</v>
       </c>
       <c r="J219" t="n">
-        <v>3383</v>
+        <v>3338</v>
       </c>
       <c r="K219" t="n">
-        <v>3662</v>
+        <v>3615</v>
       </c>
       <c r="L219" t="n">
-        <v>3970</v>
+        <v>3916</v>
       </c>
       <c r="M219" t="n">
-        <v>4139</v>
+        <v>4075</v>
       </c>
       <c r="N219" t="n">
-        <v>4216</v>
+        <v>4143</v>
       </c>
       <c r="O219" t="n">
-        <v>4322</v>
+        <v>4249</v>
       </c>
       <c r="P219" t="n">
-        <v>4391</v>
+        <v>4317</v>
       </c>
       <c r="Q219" t="n">
-        <v>4541</v>
+        <v>4467</v>
       </c>
       <c r="R219" t="n">
-        <v>4495</v>
+        <v>4397</v>
       </c>
       <c r="S219" t="n">
-        <v>4477</v>
+        <v>4351</v>
       </c>
       <c r="T219" t="n">
-        <v>4413</v>
+        <v>4278</v>
       </c>
       <c r="U219" t="n">
-        <v>4380</v>
+        <v>4242</v>
       </c>
       <c r="V219" t="n">
-        <v>4707</v>
+        <v>4526</v>
       </c>
       <c r="W219" t="n">
-        <v>4678</v>
+        <v>4504</v>
       </c>
       <c r="X219" t="n">
-        <v>4677</v>
+        <v>4504</v>
       </c>
       <c r="Y219" t="n">
-        <v>4384</v>
+        <v>4244</v>
       </c>
       <c r="Z219" t="n">
-        <v>4015</v>
+        <v>3930</v>
       </c>
       <c r="AA219" t="n">
-        <v>3673</v>
+        <v>3636</v>
       </c>
     </row>
     <row r="220">
@@ -18668,76 +18668,76 @@
         <v>11</v>
       </c>
       <c r="D220" t="n">
-        <v>3379</v>
+        <v>3291</v>
       </c>
       <c r="E220" t="n">
-        <v>3182</v>
+        <v>3118</v>
       </c>
       <c r="F220" t="n">
-        <v>3077</v>
+        <v>3028</v>
       </c>
       <c r="G220" t="n">
-        <v>3026</v>
+        <v>2984</v>
       </c>
       <c r="H220" t="n">
-        <v>3019</v>
+        <v>2978</v>
       </c>
       <c r="I220" t="n">
-        <v>3114</v>
+        <v>3073</v>
       </c>
       <c r="J220" t="n">
-        <v>3389</v>
+        <v>3346</v>
       </c>
       <c r="K220" t="n">
-        <v>3670</v>
+        <v>3624</v>
       </c>
       <c r="L220" t="n">
-        <v>3980</v>
+        <v>3928</v>
       </c>
       <c r="M220" t="n">
-        <v>4150</v>
+        <v>4089</v>
       </c>
       <c r="N220" t="n">
-        <v>4227</v>
+        <v>4157</v>
       </c>
       <c r="O220" t="n">
-        <v>4335</v>
+        <v>4265</v>
       </c>
       <c r="P220" t="n">
-        <v>4404</v>
+        <v>4332</v>
       </c>
       <c r="Q220" t="n">
-        <v>4555</v>
+        <v>4484</v>
       </c>
       <c r="R220" t="n">
-        <v>4509</v>
+        <v>4414</v>
       </c>
       <c r="S220" t="n">
-        <v>4491</v>
+        <v>4367</v>
       </c>
       <c r="T220" t="n">
-        <v>4426</v>
+        <v>4295</v>
       </c>
       <c r="U220" t="n">
-        <v>4394</v>
+        <v>4259</v>
       </c>
       <c r="V220" t="n">
-        <v>4636</v>
+        <v>4457</v>
       </c>
       <c r="W220" t="n">
-        <v>4608</v>
+        <v>4436</v>
       </c>
       <c r="X220" t="n">
-        <v>4607</v>
+        <v>4436</v>
       </c>
       <c r="Y220" t="n">
-        <v>4322</v>
+        <v>4184</v>
       </c>
       <c r="Z220" t="n">
-        <v>3962</v>
+        <v>3879</v>
       </c>
       <c r="AA220" t="n">
-        <v>3630</v>
+        <v>3594</v>
       </c>
     </row>
     <row r="221">
@@ -18751,76 +18751,159 @@
         <v>12</v>
       </c>
       <c r="D221" t="n">
-        <v>3368</v>
+        <v>3267</v>
       </c>
       <c r="E221" t="n">
-        <v>3157</v>
+        <v>3086</v>
       </c>
       <c r="F221" t="n">
-        <v>3051</v>
+        <v>3000</v>
       </c>
       <c r="G221" t="n">
-        <v>2982</v>
+        <v>2934</v>
       </c>
       <c r="H221" t="n">
-        <v>2948</v>
+        <v>2902</v>
       </c>
       <c r="I221" t="n">
-        <v>2975</v>
+        <v>2930</v>
       </c>
       <c r="J221" t="n">
-        <v>3072</v>
+        <v>3046</v>
       </c>
       <c r="K221" t="n">
-        <v>3247</v>
+        <v>3269</v>
       </c>
       <c r="L221" t="n">
-        <v>3562</v>
+        <v>3542</v>
       </c>
       <c r="M221" t="n">
-        <v>3803</v>
+        <v>3855</v>
       </c>
       <c r="N221" t="n">
-        <v>3968</v>
+        <v>4001</v>
       </c>
       <c r="O221" t="n">
-        <v>4086</v>
+        <v>4143</v>
       </c>
       <c r="P221" t="n">
-        <v>4178</v>
+        <v>4001</v>
       </c>
       <c r="Q221" t="n">
-        <v>4234</v>
+        <v>4001</v>
       </c>
       <c r="R221" t="n">
-        <v>4186</v>
+        <v>4001</v>
       </c>
       <c r="S221" t="n">
-        <v>4164</v>
+        <v>4012</v>
       </c>
       <c r="T221" t="n">
-        <v>4233</v>
+        <v>4128</v>
       </c>
       <c r="U221" t="n">
-        <v>4358</v>
+        <v>4224</v>
       </c>
       <c r="V221" t="n">
-        <v>4432</v>
+        <v>4239</v>
       </c>
       <c r="W221" t="n">
-        <v>4399</v>
+        <v>4169</v>
       </c>
       <c r="X221" t="n">
+        <v>4167</v>
+      </c>
+      <c r="Y221" t="n">
+        <v>4043</v>
+      </c>
+      <c r="Z221" t="n">
+        <v>3727</v>
+      </c>
+      <c r="AA221" t="n">
+        <v>3481</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B222" t="n">
+        <v>9</v>
+      </c>
+      <c r="C222" t="n">
+        <v>13</v>
+      </c>
+      <c r="D222" t="n">
+        <v>3198</v>
+      </c>
+      <c r="E222" t="n">
+        <v>3020</v>
+      </c>
+      <c r="F222" t="n">
+        <v>2918</v>
+      </c>
+      <c r="G222" t="n">
+        <v>2866</v>
+      </c>
+      <c r="H222" t="n">
+        <v>2845</v>
+      </c>
+      <c r="I222" t="n">
+        <v>2860</v>
+      </c>
+      <c r="J222" t="n">
+        <v>2929</v>
+      </c>
+      <c r="K222" t="n">
+        <v>3062</v>
+      </c>
+      <c r="L222" t="n">
+        <v>3363</v>
+      </c>
+      <c r="M222" t="n">
+        <v>3636</v>
+      </c>
+      <c r="N222" t="n">
+        <v>3822</v>
+      </c>
+      <c r="O222" t="n">
+        <v>4026</v>
+      </c>
+      <c r="P222" t="n">
+        <v>4115</v>
+      </c>
+      <c r="Q222" t="n">
+        <v>4080</v>
+      </c>
+      <c r="R222" t="n">
+        <v>4052</v>
+      </c>
+      <c r="S222" t="n">
+        <v>4029</v>
+      </c>
+      <c r="T222" t="n">
+        <v>4136</v>
+      </c>
+      <c r="U222" t="n">
+        <v>4239</v>
+      </c>
+      <c r="V222" t="n">
+        <v>4414</v>
+      </c>
+      <c r="W222" t="n">
         <v>4409</v>
       </c>
-      <c r="Y221" t="n">
-        <v>4124</v>
-      </c>
-      <c r="Z221" t="n">
-        <v>3784</v>
-      </c>
-      <c r="AA221" t="n">
-        <v>3526</v>
+      <c r="X222" t="n">
+        <v>4448</v>
+      </c>
+      <c r="Y222" t="n">
+        <v>4200</v>
+      </c>
+      <c r="Z222" t="n">
+        <v>3862</v>
+      </c>
+      <c r="AA222" t="n">
+        <v>3564</v>
       </c>
     </row>
   </sheetData>

</xml_diff>